<commit_message>
update study measures and probes
</commit_message>
<xml_diff>
--- a/group_membership.xlsx
+++ b/group_membership.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryantracy/Desktop/andre rc studies/police meta perceptions project/study 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4AFCA0B-41D1-694C-9927-469E9A457144}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE6E3536-826A-D941-A369-A2A47C23C230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3660" yWindow="2660" windowWidth="27640" windowHeight="16940" xr2:uid="{D84C8EAA-35AF-0C4C-8258-3A46A417A19C}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="29">
   <si>
     <t>domain</t>
   </si>
@@ -78,42 +78,6 @@
   </si>
   <si>
     <t>Extremely similar</t>
-  </si>
-  <si>
-    <t>group_membership4</t>
-  </si>
-  <si>
-    <t>To what degree do you view the typical Black police officer as an ingroup member?</t>
-  </si>
-  <si>
-    <t>group_membership5</t>
-  </si>
-  <si>
-    <t>To what degree do you think the typical Black police officer views themselves as a part of your ingroup?</t>
-  </si>
-  <si>
-    <t>group_membership6</t>
-  </si>
-  <si>
-    <t>To what degree do you view the typical Black police officer as similar to you?</t>
-  </si>
-  <si>
-    <t>group_membership7</t>
-  </si>
-  <si>
-    <t>To what degree do you view the typical White police officer as an ingroup member?</t>
-  </si>
-  <si>
-    <t>group_membership8</t>
-  </si>
-  <si>
-    <t>To what degree do you think the typical White police officer views themselves as a part of your ingroup?</t>
-  </si>
-  <si>
-    <t>group_membership9</t>
-  </si>
-  <si>
-    <t>To what degree do you view the typical White police officer as similar to you?</t>
   </si>
   <si>
     <t>group_membership10</t>
@@ -530,8 +494,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCF61DBB-4D95-9343-BB7B-9EE2889AE593}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="84.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -544,7 +511,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -561,7 +528,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
@@ -578,7 +545,7 @@
         <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="E3" t="s">
         <v>7</v>
@@ -595,7 +562,7 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
         <v>13</v>
@@ -612,7 +579,7 @@
         <v>6</v>
       </c>
       <c r="D5" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="E5" t="s">
         <v>7</v>
@@ -629,7 +596,7 @@
         <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="E6" t="s">
         <v>7</v>
@@ -646,7 +613,7 @@
         <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E7" t="s">
         <v>13</v>
@@ -663,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="E8" t="s">
         <v>7</v>
@@ -680,7 +647,7 @@
         <v>6</v>
       </c>
       <c r="D9" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="E9" t="s">
         <v>7</v>
@@ -697,111 +664,9 @@
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" t="s">
-        <v>29</v>
-      </c>
-      <c r="C12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" t="s">
-        <v>39</v>
-      </c>
-      <c r="E12" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>30</v>
-      </c>
-      <c r="B13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>40</v>
-      </c>
-      <c r="E13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" t="s">
-        <v>33</v>
-      </c>
-      <c r="C14" t="s">
-        <v>6</v>
-      </c>
-      <c r="D14" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>34</v>
-      </c>
-      <c r="B15" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>36</v>
-      </c>
-      <c r="B16" t="s">
-        <v>37</v>
-      </c>
-      <c r="C16" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" t="s">
-        <v>40</v>
-      </c>
-      <c r="E16" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>